<commit_message>
Adicionando de fato dados reais a engine, com fallback para sintetico para não quebrar
</commit_message>
<xml_diff>
--- a/data/outputs/pd_calibration_table.xlsx
+++ b/data/outputs/pd_calibration_table.xlsx
@@ -28,34 +28,34 @@
     <t>n</t>
   </si>
   <si>
-    <t>(-0.000892, 0.00106]</t>
-  </si>
-  <si>
-    <t>(0.00106, 0.0016]</t>
-  </si>
-  <si>
-    <t>(0.0016, 0.00215]</t>
-  </si>
-  <si>
-    <t>(0.00215, 0.00279]</t>
-  </si>
-  <si>
-    <t>(0.00279, 0.00356]</t>
-  </si>
-  <si>
-    <t>(0.00356, 0.00459]</t>
-  </si>
-  <si>
-    <t>(0.00459, 0.00602]</t>
-  </si>
-  <si>
-    <t>(0.00602, 0.00826]</t>
-  </si>
-  <si>
-    <t>(0.00826, 0.0127]</t>
-  </si>
-  <si>
-    <t>(0.0127, 0.189]</t>
+    <t>(-0.0009595000000000001, 0.000448]</t>
+  </si>
+  <si>
+    <t>(0.000448, 0.000723]</t>
+  </si>
+  <si>
+    <t>(0.000723, 0.00102]</t>
+  </si>
+  <si>
+    <t>(0.00102, 0.00141]</t>
+  </si>
+  <si>
+    <t>(0.00141, 0.00188]</t>
+  </si>
+  <si>
+    <t>(0.00188, 0.00253]</t>
+  </si>
+  <si>
+    <t>(0.00253, 0.00349]</t>
+  </si>
+  <si>
+    <t>(0.00349, 0.00504]</t>
+  </si>
+  <si>
+    <t>(0.00504, 0.00812]</t>
+  </si>
+  <si>
+    <t>(0.00812, 0.297]</t>
   </si>
 </sst>
 </file>
@@ -435,7 +435,7 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>0.0007143311183884485</v>
+        <v>0.0002988322343260708</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -449,10 +449,10 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>0.001319316781716872</v>
+        <v>0.0005884022195735281</v>
       </c>
       <c r="C3">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="D3">
         <v>800</v>
@@ -463,10 +463,10 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>0.001877013269831898</v>
+        <v>0.0008619744700802778</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>0.00125</v>
       </c>
       <c r="D4">
         <v>800</v>
@@ -477,10 +477,10 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>0.002463922424324868</v>
+        <v>0.001198970100863986</v>
       </c>
       <c r="C5">
-        <v>0.0025</v>
+        <v>0</v>
       </c>
       <c r="D5">
         <v>800</v>
@@ -491,10 +491,10 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>0.003162083509660011</v>
+        <v>0.001636353468765702</v>
       </c>
       <c r="C6">
-        <v>0.00375</v>
+        <v>0.00125</v>
       </c>
       <c r="D6">
         <v>800</v>
@@ -505,10 +505,10 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>0.004068664366858456</v>
+        <v>0.00220255065399456</v>
       </c>
       <c r="C7">
-        <v>0.00375</v>
+        <v>0.00625</v>
       </c>
       <c r="D7">
         <v>800</v>
@@ -519,10 +519,10 @@
         <v>10</v>
       </c>
       <c r="B8">
-        <v>0.005273724465557807</v>
+        <v>0.00297955022476534</v>
       </c>
       <c r="C8">
-        <v>0.005</v>
+        <v>0.00625</v>
       </c>
       <c r="D8">
         <v>800</v>
@@ -533,10 +533,10 @@
         <v>11</v>
       </c>
       <c r="B9">
-        <v>0.007053833263387265</v>
+        <v>0.004212424130418141</v>
       </c>
       <c r="C9">
-        <v>0.0075</v>
+        <v>0.005</v>
       </c>
       <c r="D9">
         <v>800</v>
@@ -547,10 +547,10 @@
         <v>12</v>
       </c>
       <c r="B10">
-        <v>0.01014914322035267</v>
+        <v>0.006274420765980445</v>
       </c>
       <c r="C10">
-        <v>0.0075</v>
+        <v>0.00375</v>
       </c>
       <c r="D10">
         <v>800</v>
@@ -561,10 +561,10 @@
         <v>13</v>
       </c>
       <c r="B11">
-        <v>0.02208844641898024</v>
+        <v>0.01774156875881643</v>
       </c>
       <c r="C11">
-        <v>0.02375</v>
+        <v>0.01375</v>
       </c>
       <c r="D11">
         <v>800</v>

</xml_diff>

<commit_message>
melhorando output do motor para as novas integrações com dados reais
</commit_message>
<xml_diff>
--- a/data/outputs/pd_calibration_table.xlsx
+++ b/data/outputs/pd_calibration_table.xlsx
@@ -28,34 +28,34 @@
     <t>n</t>
   </si>
   <si>
-    <t>(-0.0009595000000000001, 0.000448]</t>
-  </si>
-  <si>
-    <t>(0.000448, 0.000723]</t>
-  </si>
-  <si>
-    <t>(0.000723, 0.00102]</t>
-  </si>
-  <si>
-    <t>(0.00102, 0.00141]</t>
-  </si>
-  <si>
-    <t>(0.00141, 0.00188]</t>
-  </si>
-  <si>
-    <t>(0.00188, 0.00253]</t>
-  </si>
-  <si>
-    <t>(0.00253, 0.00349]</t>
-  </si>
-  <si>
-    <t>(0.00349, 0.00504]</t>
-  </si>
-  <si>
-    <t>(0.00504, 0.00812]</t>
-  </si>
-  <si>
-    <t>(0.00812, 0.297]</t>
+    <t>(-0.000892, 0.00106]</t>
+  </si>
+  <si>
+    <t>(0.00106, 0.0016]</t>
+  </si>
+  <si>
+    <t>(0.0016, 0.00215]</t>
+  </si>
+  <si>
+    <t>(0.00215, 0.00279]</t>
+  </si>
+  <si>
+    <t>(0.00279, 0.00356]</t>
+  </si>
+  <si>
+    <t>(0.00356, 0.00459]</t>
+  </si>
+  <si>
+    <t>(0.00459, 0.00602]</t>
+  </si>
+  <si>
+    <t>(0.00602, 0.00826]</t>
+  </si>
+  <si>
+    <t>(0.00826, 0.0127]</t>
+  </si>
+  <si>
+    <t>(0.0127, 0.189]</t>
   </si>
 </sst>
 </file>
@@ -435,7 +435,7 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>0.0002988322343260708</v>
+        <v>0.0007143311183884485</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -449,10 +449,10 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>0.0005884022195735281</v>
+        <v>0.001319316781716872</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="D3">
         <v>800</v>
@@ -463,10 +463,10 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>0.0008619744700802778</v>
+        <v>0.001877013269831898</v>
       </c>
       <c r="C4">
-        <v>0.00125</v>
+        <v>0</v>
       </c>
       <c r="D4">
         <v>800</v>
@@ -477,10 +477,10 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>0.001198970100863986</v>
+        <v>0.002463922424324868</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>0.0025</v>
       </c>
       <c r="D5">
         <v>800</v>
@@ -491,10 +491,10 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>0.001636353468765702</v>
+        <v>0.003162083509660011</v>
       </c>
       <c r="C6">
-        <v>0.00125</v>
+        <v>0.00375</v>
       </c>
       <c r="D6">
         <v>800</v>
@@ -505,10 +505,10 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>0.00220255065399456</v>
+        <v>0.004068664366858456</v>
       </c>
       <c r="C7">
-        <v>0.00625</v>
+        <v>0.00375</v>
       </c>
       <c r="D7">
         <v>800</v>
@@ -519,10 +519,10 @@
         <v>10</v>
       </c>
       <c r="B8">
-        <v>0.00297955022476534</v>
+        <v>0.005273724465557807</v>
       </c>
       <c r="C8">
-        <v>0.00625</v>
+        <v>0.005</v>
       </c>
       <c r="D8">
         <v>800</v>
@@ -533,10 +533,10 @@
         <v>11</v>
       </c>
       <c r="B9">
-        <v>0.004212424130418141</v>
+        <v>0.007053833263387265</v>
       </c>
       <c r="C9">
-        <v>0.005</v>
+        <v>0.0075</v>
       </c>
       <c r="D9">
         <v>800</v>
@@ -547,10 +547,10 @@
         <v>12</v>
       </c>
       <c r="B10">
-        <v>0.006274420765980445</v>
+        <v>0.01014914322035267</v>
       </c>
       <c r="C10">
-        <v>0.00375</v>
+        <v>0.0075</v>
       </c>
       <c r="D10">
         <v>800</v>
@@ -561,10 +561,10 @@
         <v>13</v>
       </c>
       <c r="B11">
-        <v>0.01774156875881643</v>
+        <v>0.02208844641898024</v>
       </c>
       <c r="C11">
-        <v>0.01375</v>
+        <v>0.02375</v>
       </c>
       <c r="D11">
         <v>800</v>

</xml_diff>

<commit_message>
atualizando outputs e README para realidade atual
</commit_message>
<xml_diff>
--- a/data/outputs/pd_calibration_table.xlsx
+++ b/data/outputs/pd_calibration_table.xlsx
@@ -28,34 +28,34 @@
     <t>n</t>
   </si>
   <si>
-    <t>(-0.000892, 0.00106]</t>
-  </si>
-  <si>
-    <t>(0.00106, 0.0016]</t>
-  </si>
-  <si>
-    <t>(0.0016, 0.00215]</t>
-  </si>
-  <si>
-    <t>(0.00215, 0.00279]</t>
-  </si>
-  <si>
-    <t>(0.00279, 0.00356]</t>
-  </si>
-  <si>
-    <t>(0.00356, 0.00459]</t>
-  </si>
-  <si>
-    <t>(0.00459, 0.00602]</t>
-  </si>
-  <si>
-    <t>(0.00602, 0.00826]</t>
-  </si>
-  <si>
-    <t>(0.00826, 0.0127]</t>
-  </si>
-  <si>
-    <t>(0.0127, 0.189]</t>
+    <t>(-0.0009595000000000001, 0.000448]</t>
+  </si>
+  <si>
+    <t>(0.000448, 0.000723]</t>
+  </si>
+  <si>
+    <t>(0.000723, 0.00102]</t>
+  </si>
+  <si>
+    <t>(0.00102, 0.00141]</t>
+  </si>
+  <si>
+    <t>(0.00141, 0.00188]</t>
+  </si>
+  <si>
+    <t>(0.00188, 0.00253]</t>
+  </si>
+  <si>
+    <t>(0.00253, 0.00349]</t>
+  </si>
+  <si>
+    <t>(0.00349, 0.00504]</t>
+  </si>
+  <si>
+    <t>(0.00504, 0.00812]</t>
+  </si>
+  <si>
+    <t>(0.00812, 0.297]</t>
   </si>
 </sst>
 </file>
@@ -435,7 +435,7 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>0.0007143311183884485</v>
+        <v>0.0002988322343260708</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -449,10 +449,10 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>0.001319316781716872</v>
+        <v>0.0005884022195735281</v>
       </c>
       <c r="C3">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="D3">
         <v>800</v>
@@ -463,10 +463,10 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>0.001877013269831898</v>
+        <v>0.0008619744700802778</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>0.00125</v>
       </c>
       <c r="D4">
         <v>800</v>
@@ -477,10 +477,10 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>0.002463922424324868</v>
+        <v>0.001198970100863986</v>
       </c>
       <c r="C5">
-        <v>0.0025</v>
+        <v>0</v>
       </c>
       <c r="D5">
         <v>800</v>
@@ -491,10 +491,10 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>0.003162083509660011</v>
+        <v>0.001636353468765702</v>
       </c>
       <c r="C6">
-        <v>0.00375</v>
+        <v>0.00125</v>
       </c>
       <c r="D6">
         <v>800</v>
@@ -505,10 +505,10 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>0.004068664366858456</v>
+        <v>0.00220255065399456</v>
       </c>
       <c r="C7">
-        <v>0.00375</v>
+        <v>0.00625</v>
       </c>
       <c r="D7">
         <v>800</v>
@@ -519,10 +519,10 @@
         <v>10</v>
       </c>
       <c r="B8">
-        <v>0.005273724465557807</v>
+        <v>0.00297955022476534</v>
       </c>
       <c r="C8">
-        <v>0.005</v>
+        <v>0.00625</v>
       </c>
       <c r="D8">
         <v>800</v>
@@ -533,10 +533,10 @@
         <v>11</v>
       </c>
       <c r="B9">
-        <v>0.007053833263387265</v>
+        <v>0.004212424130418141</v>
       </c>
       <c r="C9">
-        <v>0.0075</v>
+        <v>0.005</v>
       </c>
       <c r="D9">
         <v>800</v>
@@ -547,10 +547,10 @@
         <v>12</v>
       </c>
       <c r="B10">
-        <v>0.01014914322035267</v>
+        <v>0.006274420765980445</v>
       </c>
       <c r="C10">
-        <v>0.0075</v>
+        <v>0.00375</v>
       </c>
       <c r="D10">
         <v>800</v>
@@ -561,10 +561,10 @@
         <v>13</v>
       </c>
       <c r="B11">
-        <v>0.02208844641898024</v>
+        <v>0.01774156875881643</v>
       </c>
       <c r="C11">
-        <v>0.02375</v>
+        <v>0.01375</v>
       </c>
       <c r="D11">
         <v>800</v>

</xml_diff>